<commit_message>
Refresh dashboard through September 21
</commit_message>
<xml_diff>
--- a/AI-Platform-Study/dashboard/data/cochrane_dashboard_backend_template.xlsx
+++ b/AI-Platform-Study/dashboard/data/cochrane_dashboard_backend_template.xlsx
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Full-text workflow decision pending</t>
+          <t>Full-text screening underway; six oversized-PDF exceptions identified</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Screening substantially complete; decision pending for 128 studies and 3 abstracts</t>
+          <t>Full-text project active; Kate distributed all 138 available records</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Screening substantially complete; decision pending for 128 studies and 3 abstracts</t>
+          <t>Distribution succeeded; six PDFs cannot receive AI suggestions because they exceed 60 pages</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain team’s selected option and finish 3 abstracts</t>
+          <t>Document handling of the six exceptions and complete full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>TBD - after full-text set reconciliation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Full-text work held pending workflow decision</t>
+          <t>Access resolved; six-record comparability issue remains</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Substantially complete—3 abstracts pending</t>
+          <t>Restarting - commencement to be confirmed</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Decision pending for 128 studies</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Shared folder provided; PDFs being collected/uploaded for full-text screening.</t>
+          <t>Full-text package available; six PDFs exceed the Laser AI model limit</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Substantially complete—3 abstracts pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Blocked—workflow option pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Awaiting conventional export/DOIs, decision on 128 prior records, PDF-sharing method and final decision flow.</t>
+          <t>Kate distributed all 138 records; six oversized files require documented handling</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
@@ -4838,12 +4838,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Kate confirmed successful distribution of all 138 records</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4891,12 +4895,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Conventional full-text screening underway</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -4944,12 +4952,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>AI-assisted screening underway; six PDFs receive no model suggestions because they exceed 60 pages</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6633,7 +6645,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -6653,7 +6665,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Confirm logins and reviewer access before setup.</t>
+          <t>Kate confirmed that the 138 records were distributed without access issues</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -8159,7 +8171,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -12677,7 +12689,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Current shared folder in the AI Methods Group location; use this version going forward.</t>
+          <t>Repository for finalized exports and protocols; working RIS and PDF sets remain in the relevant platform until consolidation.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -12725,7 +12737,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Current source of truth. Sean updated shortcuts; the old folder should be deleted or clearly archived to avoid confusion.</t>
+          <t>Use each NK/Laser AI project as the working source; save finalized consolidated exports in this folder.</t>
         </is>
       </c>
     </row>
@@ -12996,7 +13008,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laser AI setup scheduled/confirmation pending</t>
+          <t>Setup in progress - search strategy/access issue</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -13064,7 +13076,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Documents re-forwarded; setup planned for August 18</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -13081,7 +13093,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Documents re-forwarded; setup planned for August 18</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -13098,7 +13110,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm setup, access, documents and start date</t>
+          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -13115,7 +13127,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -13132,7 +13144,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Documents re-shared; setup/access confirmation pending</t>
+          <t>Most setup materials are available; search-strategy clarification and database-access issues remain before screening can start.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -13149,7 +13161,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -13188,7 +13200,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -13270,7 +13282,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Setup scheduled for August 18; confirmation pending</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -13584,7 +13596,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress—setup confirmation pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -14545,7 +14557,7 @@
       </c>
       <c r="I63" s="18" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
@@ -14602,7 +14614,7 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J64" s="18" t="n"/>
@@ -17978,7 +17990,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -22309,7 +22321,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07; setup inputs complete and Nested Knowledge configuration underway</t>
+          <t>Converted to phase1-07; both abstract-screening arms complete</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -22324,12 +22336,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Configuration and setup validation underway</t>
+          <t>Full-text consolidation underway</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Converted to phase1-07 Human Milk; RIS, criteria, protocol information and 35 data items received</t>
+          <t>Conventional list revised to 58; AI arm completed 2,024 records; common full-text set pending</t>
         </is>
       </c>
       <c r="I12" s="17" t="inlineStr">
@@ -22413,7 +22425,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08; Laser AI setup preparation and confirmation pending</t>
+          <t>Converted to phase1-08; expected count confirmed and accessible searches received</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -22421,19 +22433,15 @@
           <t>Phase 1</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr">
-        <is>
-          <t>Syeda Kanza Naqvi / Jai Das</t>
-        </is>
-      </c>
+      <c r="F14" s="17" t="n"/>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Final upload and deduplication pending</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-08 LNS; initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending</t>
+          <t>The 14,743 count matches Covidence; seven databases were inaccessible</t>
         </is>
       </c>
       <c r="I14" s="17" t="inlineStr">
@@ -22835,7 +22843,7 @@
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Onboarding and tool training completed; awaiting final template revisions</t>
+          <t>Converted to phase1-06; screening lists reconciled and full-text screening underway</t>
         </is>
       </c>
       <c r="E28" s="17" t="inlineStr">
@@ -22850,12 +22858,12 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Awaiting final template revisions</t>
+          <t>Missing-PDF retrieval and full-text screening underway</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>Converted to phase1-06 Probiotics; Nested Knowledge allocated</t>
+          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
@@ -22939,7 +22947,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Withdrawn—conventional work completed; blinding not feasible</t>
+          <t>Team declined participation because all relevant studies had already undergone screening, INSPECT-SR, data extraction and ROB 2; blinding was not feasible.</t>
         </is>
       </c>
       <c r="E30" s="17" t="inlineStr">
@@ -22954,12 +22962,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No further action</t>
+          <t>Not participating</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Not suitable because work was already completed and blinding was impossible</t>
+          <t>Rerun search produced 377 records, but all relevant studies had already been processed. Team formally declined on 2026-08-11.</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
@@ -22969,7 +22977,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -23141,15 +23149,56 @@
       <c r="I34" s="17" t="n"/>
     </row>
     <row r="35" ht="24" customHeight="1" s="29">
-      <c r="A35" s="17" t="n"/>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="17" t="n"/>
-      <c r="E35" s="17" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="17" t="n"/>
-      <c r="H35" s="17" t="n"/>
-      <c r="I35" s="17" t="n"/>
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>new-23</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Álvaro Limones — Retention procedures for stabilising tooth position after orthodontic treatment</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Shortlisted</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>Preliminarily eligible; onboarding started</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Álvaro Limones</t>
+        </is>
+      </c>
+      <c r="G35" s="17" t="inlineStr">
+        <is>
+          <t>Searches November 2026; 300–500 references; screening and extraction December 2026</t>
+        </is>
+      </c>
+      <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t>Scope and protocol shared; schedule onboarding with the PI and review team</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="24" customHeight="1" s="29">
       <c r="A36" s="17" t="n"/>
@@ -27552,7 +27601,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Conventional screening complete; NK screening underway</t>
+          <t>Abstract sets reconciled; full-text screening underway; missing PDFs remain</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -27620,7 +27669,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Calibration and conventional screening complete; NK screening continuing</t>
+          <t>Fourteen AI-only and 16 Covidence-only records identified; common full-text pool prepared</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -27637,7 +27686,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Calibration and conventional screening complete; NK screening continuing</t>
+          <t>NK updated with the Covidence-only citations; some PDFs still need retrieval</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -27654,7 +27703,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Complete NK screening/time capture, then begin full text</t>
+          <t>Retrieve missing PDFs, complete both arms and record Bradley’s Covidence time</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -27688,7 +27737,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Conventional workflow ahead; full text awaits both workflows</t>
+          <t>Reconciliation complete; missing-PDF retrieval remains</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -27744,7 +27793,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -27843,7 +27892,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Conventional complete; NK in progress</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -27860,7 +27909,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Hold until both abstract-screening arms complete</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -27981,7 +28030,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Citations aligned; missing PDFs remain</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -28159,14 +28208,9 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Conventional complete; NK in progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -28183,7 +28227,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started—sequencing dependency</t>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Full-text lists reconciled; NK updated; missing PDFs require retrieval</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -29177,7 +29226,7 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
@@ -29230,7 +29279,7 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
@@ -29283,12 +29332,16 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>NK title/abstract output obtained and compared with Covidence</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29336,12 +29389,16 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>Both screening lists shared and reconciled</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29654,12 +29711,16 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>Common full-text pool prepared; missing PDFs still need retrieval</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29707,12 +29768,16 @@
       </c>
       <c r="I75" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J75" s="18" t="n"/>
       <c r="K75" s="18" t="n"/>
-      <c r="L75" s="18" t="n"/>
+      <c r="L75" s="18" t="inlineStr">
+        <is>
+          <t>Missing full-text PDFs are being identified and retrieved</t>
+        </is>
+      </c>
       <c r="M75" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29813,12 +29878,16 @@
       </c>
       <c r="I77" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J77" s="18" t="n"/>
       <c r="K77" s="18" t="n"/>
-      <c r="L77" s="18" t="n"/>
+      <c r="L77" s="18" t="inlineStr">
+        <is>
+          <t>Full-text comparison completed: 14 AI-only and 16 Covidence-only records</t>
+        </is>
+      </c>
       <c r="M77" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29866,12 +29935,16 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr">
+        <is>
+          <t>NK updated with the 16 Covidence-only citations</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29919,12 +29992,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Reconciled citations are ready for full-text screening</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -29977,7 +30054,11 @@
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Covidence screening underway; Bradley may assist if his time is recorded</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -30030,7 +30111,11 @@
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>NK screening underway; missing PDFs remain</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -31816,9 +31901,14 @@
           <t>task-phase1-05-003</t>
         </is>
       </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>NK and Covidence outputs received and reconciled</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -31843,9 +31933,14 @@
           <t>task-phase1-05-004</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Start onboarding only after candidate and tool are confirmed.</t>
+          <t>Reconciliation complete; retrieve missing PDFs and finish both screening arms</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -32145,7 +32240,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup confirmation pending</t>
+          <t>Both abstract-screening arms complete; full-text consolidation underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -32213,7 +32308,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Search results and data items received; awaiting setup confirmation</t>
+          <t>Conventional and AI-assisted abstract screening complete</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -32230,7 +32325,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Search results and data items received; awaiting setup confirmation</t>
+          <t>Conventional list revised to 58 references; AI arm completed 2,024 records</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -32247,7 +32342,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain setup/access/start confirmation</t>
+          <t>Correct the final NK decision, consolidate both arms and begin full-text screening</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -32264,7 +32359,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting setup confirmation</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -32281,7 +32376,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Files available; setup confirmation/document check pending</t>
+          <t>One NK decision needs correction; final common full-text set is pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -32298,7 +32393,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>Full-text setup</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -32337,7 +32432,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -32419,7 +32514,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Waiting on Meghan confirmation</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -32434,6 +32529,11 @@
           <t>abstract</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -32444,6 +32544,11 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>fullText</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -32542,7 +32647,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deduplicated search results received August 3</t>
+          <t>Deduplicated RIS/search file received - 2,053 records.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -32564,7 +32669,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Study materials collection underway</t>
+          <t>Revised 58-reference conventional list received; AI-only additions pending consolidation</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -32581,12 +32686,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Final setup-document check pending</t>
+          <t>Inclusion/exclusion criteria and PICOS received in Study Protocol Info.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -32608,7 +32713,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Selected data items received/shared</t>
+          <t>35 selected data-extraction items received.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -32625,12 +32730,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>To confirm</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Final setup-document check pending</t>
+          <t>Protocol / Study Protocol Info received.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -32727,7 +32832,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress—setup confirmation pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -32749,7 +32854,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Both abstract-screening arms completed</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -32766,7 +32876,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Under Review</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Consolidate both arms’ selections and prepare the shared full-text set</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -33678,7 +33793,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="n"/>
@@ -33788,12 +33903,16 @@
       </c>
       <c r="I65" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J65" s="18" t="n"/>
       <c r="K65" s="18" t="n"/>
-      <c r="L65" s="18" t="n"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>Murali and Michelle completed conventional abstract screening</t>
+        </is>
+      </c>
       <c r="M65" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33841,12 +33960,16 @@
       </c>
       <c r="I66" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="J66" s="18" t="n"/>
       <c r="K66" s="18" t="n"/>
-      <c r="L66" s="18" t="n"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>Mohan completed screening of 2,024 records</t>
+        </is>
+      </c>
       <c r="M66" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33894,12 +34017,16 @@
       </c>
       <c r="I67" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Needs Action</t>
         </is>
       </c>
       <c r="J67" s="18" t="n"/>
       <c r="K67" s="18" t="n"/>
-      <c r="L67" s="18" t="n"/>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>Correct the final accidentally deleted record and export the AI decisions</t>
+        </is>
+      </c>
       <c r="M67" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -33947,12 +34074,16 @@
       </c>
       <c r="I68" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J68" s="18" t="n"/>
       <c r="K68" s="18" t="n"/>
-      <c r="L68" s="18" t="n"/>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>Combine the AI and conventional full-text selections</t>
+        </is>
+      </c>
       <c r="M68" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34000,12 +34131,16 @@
       </c>
       <c r="I69" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J69" s="18" t="n"/>
       <c r="K69" s="18" t="n"/>
-      <c r="L69" s="18" t="n"/>
+      <c r="L69" s="18" t="inlineStr">
+        <is>
+          <t>Send the NK usability survey to the AI/NK reviewers, not the conventional reviewers</t>
+        </is>
+      </c>
       <c r="M69" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34265,12 +34400,16 @@
       </c>
       <c r="I74" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J74" s="18" t="n"/>
       <c r="K74" s="18" t="n"/>
-      <c r="L74" s="18" t="n"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>Revised conventional list contains 58 references; final union set pending</t>
+        </is>
+      </c>
       <c r="M74" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34477,12 +34616,16 @@
       </c>
       <c r="I78" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J78" s="18" t="n"/>
       <c r="K78" s="18" t="n"/>
-      <c r="L78" s="18" t="n"/>
+      <c r="L78" s="18" t="inlineStr">
+        <is>
+          <t>Consolidate selections from both screening arms</t>
+        </is>
+      </c>
       <c r="M78" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34530,12 +34673,16 @@
       </c>
       <c r="I79" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J79" s="18" t="n"/>
       <c r="K79" s="18" t="n"/>
-      <c r="L79" s="18" t="n"/>
+      <c r="L79" s="18" t="inlineStr">
+        <is>
+          <t>Validate the common full-text set after correcting the final NK decision</t>
+        </is>
+      </c>
       <c r="M79" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34583,12 +34730,16 @@
       </c>
       <c r="I80" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="J80" s="18" t="n"/>
       <c r="K80" s="18" t="n"/>
-      <c r="L80" s="18" t="n"/>
+      <c r="L80" s="18" t="inlineStr">
+        <is>
+          <t>Conventional reviewers may begin their 58 selections but must also screen later AI-only additions</t>
+        </is>
+      </c>
       <c r="M80" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -34636,12 +34787,16 @@
       </c>
       <c r="I81" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J81" s="18" t="n"/>
       <c r="K81" s="18" t="n"/>
-      <c r="L81" s="18" t="n"/>
+      <c r="L81" s="18" t="inlineStr">
+        <is>
+          <t>Start after the combined full-text set is finalized</t>
+        </is>
+      </c>
       <c r="M81" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -36427,9 +36582,24 @@
           <t>task-phase1-05-003</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Consolidate full-text selections and start screening</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Final-decision correction and full-text-set consolidation</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Assign one tool only after a review is selected.</t>
+          <t>Both arms completed; revised 58-reference list received; one NK decision requires correction</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -36439,7 +36609,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -36540,9 +36710,24 @@
           <t>comm-phase1-05-001</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Human Milk abstract screening complete; full-text consolidation underway</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Under Review</t>
+        </is>
+      </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>One additional eligible review still needs to be identified or confirmed for Phase 1.</t>
+          <t>Both arms completed; conventional list revised to 58; correct the final NK decision and prepare the union set</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -36824,7 +37009,6 @@
       <c r="L1" s="18" t="n"/>
       <c r="M1" s="18" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -36939,7 +37123,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation; confirmation pending</t>
+          <t>Expected reference count confirmed; available searches received</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -36990,7 +37174,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Syeda Kanza Naqvi / Jai Das</t>
+          <t>Jai Das</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -37007,7 +37191,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
+          <t>The 14,743-reference count matches Covidence; accessible searches have been supplied</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -37024,7 +37208,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
+          <t>Seven databases were inaccessible; all other search results were provided</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -37041,7 +37225,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Confirm Laser AI setup preparation, complete setup confirmation, and agree screening start plan.</t>
+          <t>Upload and deduplicate the available results; document the seven inaccessible databases</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -37058,7 +37242,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Awaiting final upload and deduplication</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -37075,7 +37259,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation is active; setup confirmation is still pending.</t>
+          <t>Count confirmed; final reference set pending incorporation of received searches</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -37092,7 +37276,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -37131,7 +37315,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -37196,7 +37380,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -37213,7 +37397,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -37228,11 +37412,6 @@
           <t>abstract</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37245,11 +37424,6 @@
           <t>fullText</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37262,11 +37436,6 @@
           <t>extraction</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -37277,11 +37446,6 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Not Started</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -37351,12 +37515,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Initial files received</t>
+          <t>Expected count confirmed; available search results received; seven databases inaccessible</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -37400,7 +37564,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Protocol/eligibility confirmation pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -37422,7 +37586,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Data items/setup confirmation pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -37444,7 +37608,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Protocol/criteria confirmation pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -37547,12 +37711,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>In Progress - setup confirmation pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Onboarding confirmed; tool allocation and setup to follow.</t>
+          <t>Count confirmed; available searches awaiting upload and deduplication</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -37575,7 +37739,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -37598,7 +37762,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -37621,7 +37785,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Withdrawn</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -37966,7 +38130,7 @@
       </c>
       <c r="I53" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J53" s="18" t="inlineStr"/>
@@ -38019,7 +38183,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J54" s="18" t="inlineStr"/>
@@ -38071,7 +38235,7 @@
       </c>
       <c r="I55" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J55" s="18" t="inlineStr"/>
@@ -38124,7 +38288,7 @@
       </c>
       <c r="I56" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J56" s="18" t="inlineStr"/>
@@ -38177,7 +38341,7 @@
       </c>
       <c r="I57" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J57" s="18" t="inlineStr"/>
@@ -38230,7 +38394,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J58" s="18" t="inlineStr"/>
@@ -38282,7 +38446,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J59" s="18" t="inlineStr"/>
@@ -38334,7 +38498,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J60" s="18" t="inlineStr"/>
@@ -38386,7 +38550,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J61" s="18" t="inlineStr"/>
@@ -38438,7 +38602,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J62" s="18" t="inlineStr"/>
@@ -38490,11 +38654,16 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J63" s="18" t="inlineStr"/>
       <c r="K63" s="18" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Available search files received; seven database searches were unavailable</t>
+        </is>
+      </c>
       <c r="M63" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -38542,12 +38711,16 @@
       </c>
       <c r="I64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J64" s="18" t="inlineStr"/>
       <c r="K64" s="18" t="inlineStr"/>
-      <c r="L64" s="18" t="inlineStr"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>Expected 14,743 count confirmed; validate final count after upload and deduplication</t>
+        </is>
+      </c>
       <c r="M64" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -41122,7 +41295,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Complete onboarding and confirm tool-training/setup plan</t>
+          <t>Incorporate the available LNS search results</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -41142,7 +41315,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>After upload and deduplication</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -41152,7 +41325,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Onboarding confirmed; tool training and setup to follow.</t>
+          <t>Count confirmed; all accessible results received; document seven inaccessible databases</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -41162,7 +41335,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -41262,37 +41435,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>LNS count confirmed; available searches received</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Krishna</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Oral galactagogues onboarding confirmed</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>Siew Cheng Foong / review team / Cochrane elective students / project team</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Krishna</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>Initial onboarding will cover the study and parallel workflow; tool training and setup will be scheduled afterward.</t>
+          <t>The count matches Covidence; available files need incorporation and deduplication</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -41652,12 +41825,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Extraction complete; Laser AI access pending</t>
+          <t>Full Blood Pressure adjudication underway; first review folder opened</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -41672,22 +41845,22 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Both workflow extractions complete; conventional files and time logs received; Laser AI outputs awaiting access</t>
+          <t>First adjudication folder shared; Bartosz completed his assessment; weekly panel meetings scheduled</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Resolve Laser AI access, download outputs and begin comparison/adjudication</t>
+          <t>Complete remaining adjudications, consolidate decisions and collect specific questions for senior reviewers</t>
         </is>
       </c>
       <c r="K4" s="22" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>Weekly through 2026-10-29</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -41724,12 +41897,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Data-extraction confirmation pending</t>
+          <t>Corrective screening in progress; consolidated full-text package available</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -41744,22 +41917,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Screening complete; awaiting final extraction files and time records</t>
+          <t>Conventional corrections received; 25-record NK corrective set ready; platform PDF package available</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Obtain final extraction files/time records and complete validation</t>
+          <t>Complete the 25-record NK screening, rerun the comparison and save the finalized export</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>Overdue / confirmation required</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -41796,7 +41969,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full-text workflow decision pending</t>
+          <t>Full-text screening underway; six-record model-limit exception open</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -41816,22 +41989,22 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Screening substantially complete; decision needed for 128 studies and final 3 abstracts</t>
+          <t>Kate distributed all 138 records; six PDFs exceed Laser AI’s 60-page limit</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Obtain team’s preferred option and complete final 3 abstracts</t>
+          <t>Resolve comparator handling for six oversized PDFs and complete both screening arms</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>TBD - after full-text set reconciliation</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -41935,7 +42108,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Laser AI setup scheduled/confirmation pending</t>
+          <t>Setup in progress - search strategy/access issue</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -41955,22 +42128,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Documents re-forwarded; setup planned for August 18</t>
+          <t>Protocol and 35 selected extraction items are received. Screening has not started. Sean is awaiting clarification on wildcard operators before executing available database searches; LILACS/IBECS access remains unresolved.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Confirm setup, access, additional documents and screening start</t>
+          <t>Clarify wildcard use, complete accessible searches, document LILACS/IBECS limitations, finalise Laser AI setup, and confirm the screening start.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -42007,7 +42180,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Broad Phase 2 deferred; one additional review onboarding separately</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -42027,17 +42200,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Planning based on results through mid-October</t>
+          <t>CD002283 is onboarding as the eighth current-study topic</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Review results after mid-October and decide next phase/tool strategy</t>
+          <t>Track CD002283 in New_Reviews until full setup begins</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>After mid-October 2026</t>
+          <t>Searches expected November 2026</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -42079,7 +42252,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Conventional abstract screening complete; NK screening underway</t>
+          <t>Abstract sets reconciled; full-text screening underway; missing PDFs remain</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -42099,12 +42272,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Calibration complete; conventional screening complete; NK screening continuing</t>
+          <t>Fourteen AI-only and 16 Covidence-only records identified; NK updated with Covidence additions</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Complete NK screening, record time and then start full text</t>
+          <t>Retrieve missing PDFs, complete both full-text arms and record Bradley’s time</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -42151,7 +42324,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nested Knowledge setup confirmation pending</t>
+          <t>Both abstract-screening arms complete; full-text consolidation underway</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -42171,22 +42344,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Search results and data items received; awaiting Meghan’s setup confirmation</t>
+          <t>Conventional arm selected 58 references; AI arm completed 2,024 records with one erroneous final decision</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Obtain setup/access/start confirmation</t>
+          <t>Correct the final NK decision, consolidate both arms’ full-text selections and send the survey to the NK reviewers</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Awaiting setup confirmation</t>
+          <t>Immediate</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -42223,7 +42396,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Laser AI setup preparation; confirmation pending</t>
+          <t>Expected 14,743-reference count confirmed; available searches received</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -42238,27 +42411,27 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Syeda Kanza Naqvi / Jai Das</t>
+          <t>Jai Das</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Initial files received; consolidated search set, protocol/eligibility, timeline and setup confirmation pending.</t>
+          <t>Count matches Covidence; all accessible searches supplied; seven databases were inaccessible</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Confirm Laser AI setup preparation, complete setup confirmation, and agree screening start plan.</t>
+          <t>Load and deduplicate the received searches, document inaccessible databases and finalize the screening set</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Setup requested 2026-08-17</t>
+          <t>Awaiting final upload and deduplication</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -45850,12 +46023,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mid April to mid-October 2026</t>
+          <t>Mid April to End June</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Laser AI continues; onboarding active</t>
+          <t>Current Focus</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -45877,12 +46050,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>July–December 2026</t>
+          <t>End June</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>In progress; CESAR-FM extension initiated</t>
+          <t>All five extension groups consented; full adjudication underway; first BP review opened and one assessment completed</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -45904,12 +46077,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Decision after mid-October results</t>
+          <t>Start July to End September</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Pending results-based decision</t>
+          <t>Broad Phase 2 deferred; CD002283 is onboarding as the eighth current-study topic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -45931,12 +46104,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>December 2026</t>
+          <t>October</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Final report/project closeout</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -46034,7 +46207,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AI Methods Group folder is the current source of truth; old folder should be archived or deleted.</t>
+          <t>Use NK/Laser AI as the working source for RIS and PDF sets; save finalized consolidated exports in this folder.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -46147,7 +46320,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Laser AI work restarted; Fruit &amp; Veg screening restart pending confirmation.</t>
+          <t>Kate distributed 138 records; six PDFs exceed the 60-page model limit and require documented comparator handling</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -46740,7 +46913,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -51505,7 +51678,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -55959,7 +56132,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Extraction complete; Laser AI access pending</t>
+          <t>Full Blood Pressure adjudication underway</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -55976,7 +56149,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -56027,7 +56200,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Both extractions complete; conventional outputs received; Laser AI retrieval pending</t>
+          <t>First adjudication review opened; weekly panel process underway</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -56044,7 +56217,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Both extractions complete; conventional outputs received; Laser AI retrieval pending</t>
+          <t>First-review folder and spreadsheet shared; Bartosz completed his assessment</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -56061,7 +56234,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Resolve access, download outputs and begin comparison</t>
+          <t>Complete remaining assessments, consolidate decisions and collect focused senior-reviewer questions</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -56078,7 +56251,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Immediate</t>
+          <t>Weekly through 2026-10-29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -56095,7 +56268,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis delayed by access</t>
+          <t>Full adjudication underway; shared senior-reviewer question document pending</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -56112,7 +56285,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Needs Action</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -56151,7 +56324,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -56284,7 +56457,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Complete—outputs submitted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -56297,11 +56470,6 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Blocked—Laser AI access pending</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -56398,7 +56566,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>All 19 records mapped; Bi 2025 supplements documented as absent from the Laser AI extraction</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -56442,7 +56610,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Conventional extraction received; Laser AI download pending</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -56481,12 +56649,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Conventional and AI time reports received</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -56559,15 +56727,11 @@
           <t>Setup / Coordination</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -56586,15 +56750,11 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -56613,15 +56773,11 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -56640,19 +56796,20 @@
           <t>Data Extraction / Analysis</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction complete; analysis access-blocked</t>
+          <t>Extraction complete; full adjudication underway</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>First BP adjudication review opened; one adjudicator completed; weekly meetings scheduled</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -59219,7 +59376,7 @@
       </c>
       <c r="I95" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J95" s="18" t="n"/>
@@ -59272,7 +59429,7 @@
       </c>
       <c r="I96" s="18" t="inlineStr">
         <is>
-          <t>Complete</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J96" s="18" t="n"/>
@@ -59325,7 +59482,7 @@
       </c>
       <c r="I97" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J97" s="18" t="n"/>
@@ -59378,7 +59535,7 @@
       </c>
       <c r="I98" s="18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J98" s="18" t="n"/>
@@ -59701,7 +59858,11 @@
       </c>
       <c r="J104" s="18" t="n"/>
       <c r="K104" s="18" t="n"/>
-      <c r="L104" s="18" t="n"/>
+      <c r="L104" s="18" t="inlineStr">
+        <is>
+          <t>Full adjudication opened; first-review materials shared and one assessment completed</t>
+        </is>
+      </c>
       <c r="M104" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -59913,7 +60074,11 @@
       </c>
       <c r="J108" s="18" t="n"/>
       <c r="K108" s="18" t="n"/>
-      <c r="L108" s="18" t="n"/>
+      <c r="L108" s="18" t="inlineStr">
+        <is>
+          <t>Weekly adjudication meetings scheduled through 29 October</t>
+        </is>
+      </c>
       <c r="M108" s="18" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -61364,7 +61529,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data-extraction confirmation pending</t>
+          <t>Corrective screening in progress; consolidated platform package available</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -61381,7 +61546,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -61432,7 +61597,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Screening complete; awaiting final extraction files and times</t>
+          <t>Full-text setup and consolidation complete; 25-record NK corrective screening remains</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -61449,7 +61614,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Screening complete; awaiting final extraction files and times</t>
+          <t>Psoriasis is currently the complete PDF package available to the extension team</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -61466,7 +61631,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Obtain final extraction files/times and complete validation</t>
+          <t>Complete the NK corrective screening, rerun the comparison and save the finalized export</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -61483,7 +61648,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Awaiting review team</t>
+          <t>Overdue / confirmation required</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -61500,7 +61665,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Final extraction completion and timing unconfirmed</t>
+          <t>Extension files are available; final validation still awaits the NK corrective decisions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -61517,7 +61682,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Waiting on Others</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -61556,7 +61721,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -61689,7 +61854,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Status requested 2026-08-17</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -61702,11 +61867,6 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>analysis</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Provisional comparison available; final validation pending</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -61803,7 +61963,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Consolidated full-text package available directly from NK; duplicate records remain documented</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -61886,12 +62046,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Screening times received; extraction time records pending</t>
+          <t>Conventional timing received: Emilie abstract 3h36m10s, full text 12h; Robin abstract 6h35m, full text 4h12m (corrected from 3h06m).</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -61992,15 +62152,11 @@
           <t>Abstract Screening</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B43" t="n">
+        <v>100</v>
+      </c>
+      <c r="C43" t="n">
+        <v>100</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -62024,15 +62180,11 @@
           <t>Full-text Screening</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="B44" t="n">
+        <v>100</v>
+      </c>
+      <c r="C44" t="n">
+        <v>100</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -62041,7 +62193,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Conventional and AI-assisted full-text screening complete; 10 studies selected.</t>
+          <t>Full-text package consolidated for export; the 25-record NK corrective screening remains pending</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -62064,7 +62216,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Extraction status awaiting review team</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -64636,7 +64788,7 @@
       </c>
       <c r="I95" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J95" s="18" t="n"/>
@@ -64689,7 +64841,7 @@
       </c>
       <c r="I96" s="18" t="inlineStr">
         <is>
-          <t>Under Review</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J96" s="18" t="n"/>

</xml_diff>